<commit_message>
Show every source table each scenario's target depends on
Four tabs showed a target row carrying a value with no visible source.
S03 omitted SRC_1 entirely, though its target carries A1. S06 omitted
SRC_1 on Day 1 and SRC_2 throughout. S07 omitted SRC_1. S08 omitted
SRC_2.

Each now shows both source tables, and where a source does not move
between Day 1 and Day 2 it is shown again, greyed, marked unchanged -
rather than left out. S01's Day 2 gains the same treatment: SRC_1
standing still is the whole point of that scenario, so it is now a
table rather than a remark in a heading.

Checked the rest of the workbook the same way: no tab now shows a
target value whose source table is absent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCJmVmyRxrvx1fnzSrSCBX
</commit_message>
<xml_diff>
--- a/w3-scd-effective-date-split/SCD2_Scenarios.xlsx
+++ b/w3-scd-effective-date-split/SCD2_Scenarios.xlsx
@@ -87,17 +87,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F7E2DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCF3E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -146,11 +146,11 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -600,7 +600,7 @@
           <t>The core problem. Also the only scenario that fires BOTH retirement mechanisms</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Proven (dead-record half needs re-run)</t>
         </is>
@@ -627,7 +627,7 @@
           <t>Assumed to be the hard case; it is not</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Covered, not separately tested</t>
         </is>
@@ -735,7 +735,7 @@
           <t>Dates alone cannot tell old from new</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Proven (as dead record, needs re-run)</t>
         </is>
@@ -762,7 +762,7 @@
           <t>Restatements, or distinct versions? Changes the design</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>OPEN — Q1, Q2</t>
         </is>
@@ -870,7 +870,7 @@
           <t>Update in place, or one rule always?</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>OPEN DECISION — Q3</t>
         </is>
@@ -897,14 +897,14 @@
           <t>The only case where ABC writes to our target</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>NOT TESTED — Q4</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Not covered by a scenario tab — no data needed</t>
         </is>
@@ -926,79 +926,79 @@
       <c r="E20" s="4" t="inlineStr"/>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="11" t="inlineStr"/>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>SCD2 + SCD1 → SCD2   /   SCD2 + lookup → SCD2</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr"/>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>The SCD2 table sets the dates on its own. This is today's established pattern, no new logic</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr"/>
+      <c r="E21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="11" t="inlineStr"/>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>SCD1 + SCD1 → SCD2</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr"/>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Neither source carries history; target dates come from the load date</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr"/>
+      <c r="E22" s="7" t="inlineStr"/>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="11" t="inlineStr"/>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr"/>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>SCD2 + SCD2 → SCD1</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr"/>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>No history to keep in the target — take the latest value</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr"/>
+      <c r="E23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="11" t="inlineStr"/>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr"/>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Historical / catchup / first-time-incremental load</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr"/>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>ABC has not built these execution types yet</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr"/>
+      <c r="E24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="11" t="inlineStr"/>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr"/>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Mixed clocks: one source load-timed, one business-timed</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr"/>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Confirmed limitation. A decision to take, not a case to test</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr"/>
+      <c r="E25" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1233,28 +1233,28 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>•  There is nothing in the target to compare against, so every interval is an insert and nothing is retired.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>•  No special first-load path is needed — it is the ordinary logic with an empty target.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -1345,28 +1345,28 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>•  This is the baseline. See tab S01 for the worked data.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>•  Everything in Group A (S01 to S09) assumes execution_type = NEW.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -1501,37 +1501,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>K1</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>the existing row's expiry is EDITED. 1 row. No record it ever said 9999.</t>
         </is>
@@ -1656,35 +1656,35 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>•  Our comparison is content-based, not timestamp-based. A Zone 1 rerun that changes nothing already produces ZERO rows on its own — no branch required to achieve that.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>•  The framework's own MERGE does need the branch, because it is row-by-row and on a Z1 rerun every record gets a new refined timestamp and a new UUID, so everything lands in the delta and has to be absorbed as an update. That reasoning does not carry over to this design.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>•  Cost of Option A: the target's contents depend on HOW the run was triggered rather than on what the data says. The same source data loaded two ways gives two different tables, and you would need the run history to explain the difference.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
@@ -1712,28 +1712,28 @@
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Do we branch on execution_type at all, or apply one rule always?</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr"/>
-      <c r="D22" s="10" t="inlineStr"/>
-      <c r="E22" s="10" t="inlineStr"/>
-      <c r="F22" s="10" t="inlineStr"/>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr"/>
+      <c r="D22" s="11" t="inlineStr"/>
+      <c r="E22" s="11" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr"/>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>My recommendation is one rule always (Option B). Overrule me if the framework requires the update-in-place shape for a reason we have not found.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -1862,87 +1862,87 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>K1</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>retired by run 102</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>K1</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>dead record, by run 102</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr"/>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr"/>
+      <c r="B8" s="8" t="inlineStr"/>
+      <c r="C8" s="8" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>*** run fails here — none of the 4 inserts happened ***</t>
         </is>
@@ -1973,83 +1973,83 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr"/>
-      <c r="F12" s="10" t="inlineStr"/>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>DELETE the rows the failed run inserted, found by execution_run_id + job_run_id</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr"/>
-      <c r="E13" s="10" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr"/>
+      <c r="D13" s="11" t="inlineStr"/>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>UN-EXPIRE the rows the failed run expired, same key</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>•  Step 1 of the cleanup works — our inserted rows do carry run 102.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>•  Step 2 does NOT work. Our retired rows still carry the run id of the run that INSERTED them (run 101), not the run that retired them (102). The cleanup cannot find them.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>•  Net effect: the new rows are deleted, the old ones stay retired, and the key now has a HOLE in its timeline.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>•  The restart should then recompute from scratch, see the hole, and refill it — so it probably self-heals. 'Probably' is doing a lot of work in that sentence and this is untested.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>•  Cheapest fix if we need one: stamp the retiring run's id onto the row in the retirement step.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
@@ -2077,28 +2077,28 @@
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Does ABC's automatic target cleanup run against this target, and can we opt out of it?</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr"/>
-      <c r="D24" s="10" t="inlineStr"/>
-      <c r="E24" s="10" t="inlineStr"/>
-      <c r="F24" s="10" t="inlineStr"/>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr"/>
+      <c r="D24" s="11" t="inlineStr"/>
+      <c r="E24" s="11" t="inlineStr"/>
+      <c r="F24" s="11" t="inlineStr"/>
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>If it runs, we should test the failure above rather than assume it self-heals.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -2210,23 +2210,23 @@
       </c>
     </row>
     <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Multiple rows for the same (key, effective date) in one window — restatements where the latest wins, or distinct versions that must all be loaded?</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>We keep only the latest. If all must load, two live rows would share a key and effective date and the timeline becomes ambiguous.</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
@@ -2427,7 +2427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2750,7 +2750,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>DAY 2 — SRC_2 changes.  SRC_1 IS NOT TOUCHED.</t>
+          <t>DAY 2 — SRC_1  (UNCHANGED — no new row, no closed row)</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_2</t>
+          <t>NON_KEY_1</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2777,11 +2777,8 @@
       </c>
       <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>WHAT CHANGED</t>
-        </is>
-      </c>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2791,26 +2788,27 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr"/>
       <c r="F21" s="7" t="inlineStr"/>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>closed early — was 9999-12-31</t>
-        </is>
-      </c>
+          <t>same as Day 1</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2820,282 +2818,192 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>9999-12-31</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr"/>
       <c r="F22" s="7" t="inlineStr"/>
       <c r="G22" s="7" t="inlineStr">
         <is>
+          <t>same as Day 1</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — SRC_2 changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>WHAT CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>closed early — was 9999-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr"/>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
           <t>new version</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>K1</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>new version</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>DAY 2 — TGT  (7 rows)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>PRIMARY_KEY</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>NON_KEY_1</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>NON_KEY_2</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>ROW_EFF_DATE</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>DELETE_IND</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>ACTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>RETIRED — exp was a real date, so delete indicator</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>DEAD RECORD — exp was 9999, so exp pulled back to its own eff date</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>insert</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>insert</t>
         </is>
       </c>
     </row>
@@ -3107,22 +3015,22 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -3132,7 +3040,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>insert</t>
+          <t>untouched</t>
         </is>
       </c>
     </row>
@@ -3144,143 +3052,328 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>RETIRED — exp was a real date, so delete indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>DEAD RECORD — exp was 9999, so exp pulled back to its own eff date</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>insert</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>insert</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>insert</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>insert</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>•  SRC_1 never changed on Day 2, yet TWO of its three target rows had to be retired. Neither source on its own can decide the target's dates — this is the whole problem in one picture.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>•  How the target rows are derived: collect every date either source mentions (09, 10, 15, 21, 22, 9999), then every consecutive pair of dates becomes one target row, filled from whichever source version covers it.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>•  This one scenario fires BOTH retirement mechanisms, which is why it is the base example:</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="9" t="inlineStr">
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>•       A1|B1|10-Sep→21-Sep  had a real expiry date  →  DELETE_IND = 'Y', dates left alone.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>•       A2|B1|21-Sep→9999    had the high end date   →  DEAD RECORD, expiry pulled back to 21-Sep so the row spans zero days.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>•  The dead record and the new A2|B2|21-Sep row share an effective date. That is fine — the dead one covers no time, so no as-of query can return it.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>•  The first target row carries a blank NON_KEY_1 because SRC_2 starts on 09-Sep but SRC_1 does not start until 10-Sep. We keep the row rather than dropping it.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr"/>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
-      <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="inlineStr"/>
-      <c r="G45" s="5" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="5" t="inlineStr"/>
-      <c r="C46" s="5" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr"/>
-      <c r="E46" s="5" t="inlineStr"/>
-      <c r="F46" s="5" t="inlineStr"/>
-      <c r="G46" s="5" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr"/>
-      <c r="B47" s="5" t="inlineStr"/>
-      <c r="C47" s="5" t="inlineStr"/>
-      <c r="D47" s="5" t="inlineStr"/>
-      <c r="E47" s="5" t="inlineStr"/>
-      <c r="F47" s="5" t="inlineStr"/>
-      <c r="G47" s="5" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr"/>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="5" t="inlineStr"/>
-      <c r="G48" s="5" t="inlineStr"/>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A43:G43"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3550,58 +3643,58 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>closed early</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>new version</t>
         </is>
@@ -3644,58 +3737,58 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>closed early</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr"/>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>new version</t>
         </is>
@@ -3894,28 +3987,28 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>•  No different in kind from S01. Dates from both sides go into the same pot before the intervals are cut, so it does not matter whether one source moved or both.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>•  Listed separately only because this is the case people assume is the hardest, and it is not.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -3972,7 +4065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4001,7 +4094,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DAY 1 — SRC_2  (NOTE_TEXT is NOT carried to the target)</t>
+          <t>DAY 1 — SRC_1</t>
         </is>
       </c>
     </row>
@@ -4013,24 +4106,20 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_2</t>
+          <t>NON_KEY_1</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>NOTE_TEXT</t>
+          <t>ROW_EFF_DATE</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ROW_EFF_DATE</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
     </row>
@@ -4042,31 +4131,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
           <t>9999-12-31</t>
         </is>
       </c>
+      <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>DAY 1 — TGT</t>
+          <t>DAY 1 — SRC_2  (NOTE_TEXT is NOT carried to the target)</t>
         </is>
       </c>
     </row>
@@ -4078,12 +4163,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_1</t>
+          <t>NON_KEY_2</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_2</t>
+          <t>NOTE_TEXT</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -4096,58 +4181,42 @@
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>DELETE_IND</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>ACTION</t>
-        </is>
-      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>K3</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>insert</t>
-        </is>
-      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>DAY 2 — SRC_2 splits, but only NOTE_TEXT differs</t>
+          <t>DAY 1 — TGT</t>
         </is>
       </c>
     </row>
@@ -4159,254 +4228,398 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>NON_KEY_1</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>NON_KEY_2</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>DELETE_IND</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>ACTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>insert</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — SRC_1  (UNCHANGED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_1</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>same as Day 1</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — SRC_2 splits, but only NOTE_TEXT differs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>NOTE_TEXT</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>ROW_EFF_DATE</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>WHAT CHANGED</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>K3</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>original</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>closed early</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>K3</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>reworded</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>new version — NON_KEY_2 is still B1</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>DAY 2 — TGT</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>PRIMARY_KEY</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>NON_KEY_1</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>NON_KEY_2</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>ROW_EFF_DATE</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>DELETE_IND</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>ACTION</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>K3</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>NO CHANGE — 0 rows written</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>•  Before any dates are collected, each source is cut down to only the columns that actually reach the target, then consecutive identical versions are merged back together.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>•  The 12-Jul boundary disappears before it can split anything, so the target is untouched.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>•  Without this step the target would gain a split into two IDENTICAL rows — a change that means nothing to any consumer, and one that would then have to be undone.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr"/>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr"/>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="5" t="inlineStr"/>
-      <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="5" t="inlineStr"/>
-      <c r="F29" s="5" t="inlineStr"/>
-      <c r="G29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A30:G30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4808,183 +5021,183 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>WRONG — A1 merged into 01-Mar→9999, so it overlaps A2</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>duplicate period</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>•  The two A1 runs must stay SEPARATE. If they are merged because the value matches, you get one A1 version spanning 01-Mar to 9999 which overlaps the A2 version.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>•  The middle interval then matches TWO source versions instead of one, and the join produces duplicate target rows.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>•  Rule: only CONSECUTIVE identical versions merge — never any two that happen to have the same value.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -5407,72 +5620,72 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>K5</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>WRONG — the two A1 versions merged, so 10-Apr and 20-Apr vanished and the target now claims cover the source never gave</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>•  The source says nothing at all about 10-Apr to 20-Apr, so the target must say nothing either — the middle row carries a blank rather than being filled in or dropped.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>•  The two A1 versions must NOT merge across the gap even though the value is identical. A gap is not a match.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>•  This is why the date collection uses expiry dates as well as effective dates. Using only effective dates would lose both boundaries.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
@@ -5530,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5559,7 +5772,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DAY 1 — TGT holds</t>
+          <t>DAY 1 — SRC_1</t>
         </is>
       </c>
     </row>
@@ -5576,71 +5789,47 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_2</t>
+          <t>ROW_EFF_DATE</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ROW_EFF_DATE</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>DELETE_IND</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>ACTION</t>
-        </is>
-      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>K6</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>insert</t>
-        </is>
-      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>DAY 2 — SRC_1 restates the SAME row with a different value.  BOTH DATES ARE UNCHANGED.</t>
+          <t>DAY 1 — SRC_2</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5841,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_1</t>
+          <t>NON_KEY_2</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -5667,45 +5856,37 @@
       </c>
       <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>WHAT CHANGED</t>
-        </is>
-      </c>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>K6</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>A9</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>value A1 → A9. Dates identical.</t>
-        </is>
-      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>DAY 2 — TGT</t>
+          <t>DAY 1 — TGT</t>
         </is>
       </c>
     </row>
@@ -5747,147 +5928,356 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>K6</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>insert</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — SRC_1 restates the SAME row with a different value.  BOTH DATES ARE UNCHANGED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_1</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>WHAT CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>value A1 → A9. Dates identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — SRC_2  (UNCHANGED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>same as Day 1</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>DAY 2 — TGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_1</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>DELETE_IND</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>ACTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>DEAD RECORD — exp was 9999</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>K6</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>A9</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>insert</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>•  The dates alone cannot tell the old row from the new one — they are identical. The comparison therefore includes a hash of the values carried to the target, not just the two dates.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>•  If the comparison used dates only: old matches new, nothing is written, the stale A1 stays in the target permanently, and the job reports success. A silent failure.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr"/>
-      <c r="G23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr"/>
-      <c r="G25" s="5" t="inlineStr"/>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A30:G30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5899,7 +6289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5928,7 +6318,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SRC_2 — two rows with the SAME key and SAME effective date, inside one sourcing window</t>
+          <t>SRC_1  (one version, unchanged — it is SRC_2 that arrives twice)</t>
         </is>
       </c>
     </row>
@@ -5940,7 +6330,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>NON_KEY_2</t>
+          <t>NON_KEY_1</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -5953,157 +6343,133 @@
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>REFINED_TIMESTAMP</t>
-        </is>
-      </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>K7</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>SRC_2 — two rows with the SAME key and SAME effective date, inside one sourcing window</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>REFINED_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>K7</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>2026-09-22 08:00</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr"/>
-      <c r="G6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>K7</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>2026-09-22 14:00</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>OPTION (a) — they are RESTATEMENTS, latest wins   [what we built today]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>PRIMARY_KEY</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>NON_KEY_1</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>NON_KEY_2</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>ROW_EFF_DATE</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>ROW_EXP_DATE</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>DELETE_IND</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>ACTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>K7</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>the 14:00 row wins, the 08:00 row is discarded</t>
-        </is>
-      </c>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>OPTION (b) — they are DISTINCT versions, both must land</t>
+          <t>OPTION (a) — they are RESTATEMENTS, latest wins   [what we built today]</t>
         </is>
       </c>
     </row>
@@ -6145,225 +6511,306 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>K7</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>the 14:00 row wins, the 08:00 row is discarded</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>OPTION (b) — they are DISTINCT versions, both must land</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_1</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>DELETE_IND</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>ACTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>K7</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>K7</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>? — two LIVE rows share a key and effective date. The timeline is now ambiguous.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>•  Our current logic keeps only the LATEST refined timestamp per (key, effective date). That is correct if the second row is a restatement of the first.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>•  You said these 'need to get loaded in zone2 target'. If ALL of them must land, our logic is dropping data you want.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>•  Under option (b) the target ends up with two live rows sharing a key and effective date, which breaks the timeline — UNLESS the effective date carries a time component, in which case they never collide and nothing special is needed.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>QUESTION</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>WHY IT MATTERS / MY VIEW</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="29" ht="46" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Are multiple rows for the same (key, effective date) in one window RESTATEMENTS (latest wins) or DISTINCT versions that must all be loaded?</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr"/>
-      <c r="D25" s="10" t="inlineStr"/>
-      <c r="E25" s="10" t="inlineStr"/>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr"/>
+      <c r="D29" s="11" t="inlineStr"/>
+      <c r="E29" s="11" t="inlineStr"/>
+      <c r="F29" s="11" t="inlineStr"/>
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>This is the one that could change the design rather than just the documentation.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Is ROW_EFF_DATE a DATE or a TIMESTAMP?</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr"/>
-      <c r="D26" s="10" t="inlineStr"/>
-      <c r="E26" s="10" t="inlineStr"/>
-      <c r="F26" s="10" t="inlineStr"/>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr"/>
+      <c r="E30" s="11" t="inlineStr"/>
+      <c r="F30" s="11" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>If intraday runs produce different times, option (b) resolves itself and there is no conflict at all.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="5" t="inlineStr"/>
-      <c r="F29" s="5" t="inlineStr"/>
-      <c r="G29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr"/>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="5" t="inlineStr"/>
-      <c r="G32" s="5" t="inlineStr"/>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6375,7 +6822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6404,7 +6851,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SRC_1 and SRC_2 — K8's rows were last refined before this run's window</t>
+          <t>SRC_1 — last refined long before this run's sourcing window</t>
         </is>
       </c>
     </row>
@@ -6434,34 +6881,34 @@
       <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>K8</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr"/>
-      <c r="F6" s="11" t="inlineStr"/>
-      <c r="G6" s="11" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>SRC_2 — same, untouched this run</t>
         </is>
       </c>
     </row>
@@ -6473,140 +6920,197 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>NON_KEY_2</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EFF_DATE</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>ROW_EXP_DATE</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>K8</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>9999-12-31</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>PRIMARY_KEY</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>NON_KEY_1</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>NON_KEY_2</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>ROW_EFF_DATE</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>ROW_EXP_DATE</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>DELETE_IND</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>ACTION</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>K8</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>9999-12-31</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>NO CHANGE — key never enters the run</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>How this works</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>•  K8 is not read and not written. It never appears in the list of impacted keys, so no work is done for it at all.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>•  This is what keeps the run proportional to what actually changed rather than to the size of the table.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Your comments</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr"/>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>